<commit_message>
chore: remove outdated report for electricity prices on 08.09.2026
</commit_message>
<xml_diff>
--- a/Historico_Precios_Cierre_Mercado_Futuros_Energía Eléctrica.xlsx
+++ b/Historico_Precios_Cierre_Mercado_Futuros_Energía Eléctrica.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\PRECIOS MERCADO\Precio diario\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC41\Desktop\Dev\Informe Diario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5C65FB-6022-4F4B-A43A-AF2D9783A160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E2AFBB2-A07B-4126-9A6B-AE08EC12FDAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{76DFC19C-C10A-4D0D-BC63-26CAA662C9B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{76DFC19C-C10A-4D0D-BC63-26CAA662C9B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Q1 " sheetId="3" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="11">
   <si>
     <t>Fecha</t>
   </si>
@@ -240,9 +240,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -280,7 +280,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -386,7 +386,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -528,7 +528,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9147,32 +9147,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
-      <c r="A2" s="2">
-        <v>46108</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="4">
-        <v>86.25</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A3" s="2">
-        <v>46024</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="4">
-        <v>66.3</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1">
       <c r="A4" s="2"/>

</xml_diff>